<commit_message>
August update with new labels and corrections.
</commit_message>
<xml_diff>
--- a/IEDC_Classification_fill/manual_insert/IEDC_100_NZIA_final_products.xlsx
+++ b/IEDC_Classification_fill/manual_insert/IEDC_100_NZIA_final_products.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10402"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC3E0E4-141F-4D5C-905C-9F72610EB5DB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7945122A-44F7-9F48-9E46-B91B1793B586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-1960" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definition" sheetId="2" r:id="rId1"/>
@@ -16,12 +16,22 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="87">
   <si>
     <t>Column</t>
   </si>
@@ -200,18 +210,9 @@
     <t>Extracted from the EU COMMISSION IMPLEMENTING REGULATION (EU) 2025/1178 of 23 May 2025</t>
   </si>
   <si>
-    <t>Solar PV systems</t>
-  </si>
-  <si>
     <t>attribute5_anc</t>
   </si>
   <si>
-    <t>Photovoltaic (PV) technologies</t>
-  </si>
-  <si>
-    <t>Solar technologies</t>
-  </si>
-  <si>
     <t>NZIA_final_products</t>
   </si>
   <si>
@@ -227,17 +228,77 @@
     <t>final product as listed by the NZIA (or amended from other sources)</t>
   </si>
   <si>
-    <t>Concentrated solar power (CSP) plants</t>
-  </si>
-  <si>
-    <t>Solar thermal electric technologies</t>
+    <t>solar technology</t>
+  </si>
+  <si>
+    <t>photovoltaic (PV) technologies</t>
+  </si>
+  <si>
+    <t>tunnel oxide passivated contact solar cells (TOPCon)</t>
+  </si>
+  <si>
+    <t>silicon heterojunction solar cells (SHJ)</t>
+  </si>
+  <si>
+    <t>perovskite silicon tandem solar cells (PST)</t>
+  </si>
+  <si>
+    <t>battery and energy storage technologies</t>
+  </si>
+  <si>
+    <t>battery technologies</t>
+  </si>
+  <si>
+    <t>nickel manganese cobalt lithium-ion batteries (NMC)</t>
+  </si>
+  <si>
+    <t>lithium iron phosphate batteries (LFP)</t>
+  </si>
+  <si>
+    <t>lithium manganese iron phosphate batteries (LMFP)</t>
+  </si>
+  <si>
+    <t>sodium-ion batteries (SIB)</t>
+  </si>
+  <si>
+    <t>onshore and offshore wind energy technologies</t>
+  </si>
+  <si>
+    <t>wind turbine technologies</t>
+  </si>
+  <si>
+    <t>wind turbines, onshore and offshore</t>
+  </si>
+  <si>
+    <t>hydrogen technologies</t>
+  </si>
+  <si>
+    <t>electrolyzer technologies</t>
+  </si>
+  <si>
+    <t>alkaline electrolyzers (AEL)</t>
+  </si>
+  <si>
+    <t>proton exchange membrane  electrolyzers (PEMEL)</t>
+  </si>
+  <si>
+    <t>anion exchange membrane electrolyzers (AEMEL)</t>
+  </si>
+  <si>
+    <t>solid-oxide electrolyzers (SOEL)</t>
+  </si>
+  <si>
+    <t>wind turbines, onshore</t>
+  </si>
+  <si>
+    <t>wind turbines, offshore</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -263,6 +324,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -301,22 +368,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -599,13 +658,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.578125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -616,45 +675,45 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>100</v>
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>64</v>
+      <c r="B5" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -663,25 +722,25 @@
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -690,16 +749,16 @@
       </c>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -710,168 +769,168 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="3"/>
+      <c r="B13" s="2"/>
       <c r="C13" s="2"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+        <v>63</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="3"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="2"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="3"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="3"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="2"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C18" s="2"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C20" s="2"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C21" s="2"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="3"/>
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="3"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="3"/>
+      <c r="B24" s="2"/>
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="3"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="3"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="2"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="3"/>
+      <c r="B27" s="2"/>
       <c r="C27" s="2"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="3"/>
+      <c r="B28" s="2"/>
       <c r="C28" s="2"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
+      <c r="B29" s="2"/>
       <c r="C29" s="2"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="3"/>
+      <c r="B30" s="2"/>
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>57</v>
       </c>
       <c r="C31" s="2"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="4">
         <v>45847</v>
       </c>
       <c r="C32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C33" s="2"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>2</v>
       </c>
@@ -880,12 +939,12 @@
       </c>
       <c r="C34" s="2"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -897,54 +956,54 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.05078125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:T23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="8.578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20.41796875" customWidth="1"/>
-    <col min="9" max="9" width="10.734375" customWidth="1"/>
-    <col min="10" max="10" width="18.15625" customWidth="1"/>
-    <col min="11" max="11" width="24.7890625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.05078125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" customWidth="1"/>
+    <col min="10" max="10" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>43</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="K1" s="11" t="s">
+      <c r="J1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="1" t="s">
         <v>46</v>
       </c>
       <c r="M1" s="1" t="s">
@@ -972,7 +1031,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -983,16 +1042,13 @@
         <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="J2" t="s">
-        <v>61</v>
-      </c>
-      <c r="K2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1003,115 +1059,354 @@
         <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="J3" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
-      <c r="F4" s="8"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
         <v>100</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
         <v>100</v>
       </c>
-    </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F39" s="9"/>
-    </row>
-    <row r="40" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F40" s="9"/>
-    </row>
-    <row r="41" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F41" s="9"/>
-    </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F42" s="9"/>
-    </row>
-    <row r="43" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F43" s="9"/>
-    </row>
-    <row r="44" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F44" s="9"/>
-    </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F45" s="9"/>
-    </row>
-    <row r="46" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F46" s="10"/>
-    </row>
-    <row r="47" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F47" s="9"/>
-    </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F48" s="10"/>
-    </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F49" s="10"/>
-    </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F50" s="10"/>
-    </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F51" s="10"/>
-    </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F52" s="10"/>
-    </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F53" s="10"/>
-    </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F54" s="10"/>
-    </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F55" s="10"/>
-    </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F56" s="10"/>
-    </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F57" s="10"/>
-    </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F58" s="10"/>
-    </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F59" s="10"/>
-    </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="F60" s="10"/>
+      <c r="E7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" t="s">
+        <v>75</v>
+      </c>
+      <c r="J7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>100</v>
+      </c>
+      <c r="E8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>100</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>66</v>
+      </c>
+      <c r="J9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>100</v>
+      </c>
+      <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>100</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+      <c r="E12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" t="s">
+        <v>69</v>
+      </c>
+      <c r="J12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>100</v>
+      </c>
+      <c r="E13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>100</v>
+      </c>
+      <c r="E14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="J14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>100</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="J15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>86</v>
+      </c>
+      <c r="J16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>100</v>
+      </c>
+      <c r="E17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" t="s">
+        <v>78</v>
+      </c>
+      <c r="J17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>100</v>
+      </c>
+      <c r="E18" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+      <c r="J18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>13</v>
+      </c>
+      <c r="B19">
+        <v>100</v>
+      </c>
+      <c r="E19" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+      <c r="J19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>13</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
+      </c>
+      <c r="E20" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" t="s">
+        <v>81</v>
+      </c>
+      <c r="J20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>13</v>
+      </c>
+      <c r="B21">
+        <v>100</v>
+      </c>
+      <c r="E21" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" t="s">
+        <v>82</v>
+      </c>
+      <c r="J21" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>13</v>
+      </c>
+      <c r="B22">
+        <v>100</v>
+      </c>
+      <c r="E22" t="s">
+        <v>58</v>
+      </c>
+      <c r="F22" t="s">
+        <v>83</v>
+      </c>
+      <c r="J22" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>100</v>
+      </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" t="s">
+        <v>84</v>
+      </c>
+      <c r="J23" t="s">
+        <v>79</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>